<commit_message>
update: perbaikan algoritma GA / fitur baru
</commit_message>
<xml_diff>
--- a/backend/aes_baseline_history.xlsx
+++ b/backend/aes_baseline_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1067,7 +1067,110 @@
           <t>0.18926667807329142</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-04-25 02:04:32</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>PDF_Deid_Deidentification_0.pdf</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>28.80</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.8132</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>7.994089607585593</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Lolos</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Lolos</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>0.9967162834555253</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.2154279082024675</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-04-25 05:44:46</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AES-128-GA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PDF_Deid_Deidentification_2.pdf</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>28.54</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1a977e195860b8727fa3b7e7cde4c5c2</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0.7377</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0.74</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>7.995061520966284</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Lolos</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Lolos</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>0.5598289264530043</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.5821186815772154</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Perubahan pada history dan Ga_Keygen
</commit_message>
<xml_diff>
--- a/backend/aes_baseline_history.xlsx
+++ b/backend/aes_baseline_history.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -429,6 +429,8 @@
     <col width="22" customWidth="1" min="11" max="11"/>
     <col width="22" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -494,6 +496,16 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>ber_value</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>ber_percentage</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>catatan</t>
         </is>
       </c>
@@ -501,7 +513,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-05-07 17:38:40</t>
+          <t>2026-05-11 04:59:48</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,51 +523,1213 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>PDF_Deid_Deidentification_2.pdf</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>38.14</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>35FCA34ED29D577E5536EC2AB112925E</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>0.8042</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-05-11 05:00:18</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>PDF_Deid_Deidentification_2.pdf</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>28.54</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>35FCA34ED29D577E5536EC2AB112925E</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>0.8042</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>0.4289</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>7.995140372449971</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Lolos</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lolos</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0.3711515319804682</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.8289350997598831</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-05-14 16:17:59</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>PDF_Deid_Deidentification_0.pdf</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D4" t="n">
         <v>38.48</v>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>4045742093B3F45EFDCA3B8230C37F6A</t>
         </is>
       </c>
-      <c r="F2" t="n">
-        <v>2.1607</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>0.9167</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:30:14</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Data_Uji_2.pdf</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>28.54</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>53755C186CF0CCBA52B29573D05FC676</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9964</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:30:52</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Data_Uji_3.pdf</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>28.54</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>35FCA34ED29D577E5536EC2AB112925E</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>0.5741000000000001</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:31:21</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Data_Uji_5.pdf</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>28.61</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>09097C7A47328F7692E327F42093AD61</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>0.4247</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:31:42</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Data_Uji_1.pdf</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>4045742093B3F45EFDCA3B8230C37F6A</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.4746</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:31:46</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Data_Uji_4.pdf</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>28.81</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CB11DF880FD86805A16083F05A0983B6</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:32:58</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Data_Uji_4_Sedang.pdf</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>249.82</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>B6F626ACC56BD68776D852561AED813E</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>3.3286</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:33:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Data_Uji_5_Sedang.pdf</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>250.35</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>C05840FBE2AC5615186C9338E875B2B7</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>2.3333</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:33:03</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Data_Uji_2_Sedang.pdf</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>258.49</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>CC12011C235919D1AB88C4BDFBAD838D</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>3.7398</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:33:06</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Data_Uji_3_Sedang.pdf</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>260.82</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>41188A2C22997A95A487B7653FE5642E</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>3.0667</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:33:09</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Data_Uji_1_Sedang.pdf</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>266.73</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>B44A88F269DF6071532F3E02F930BC52</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3.91</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-05-15 14:33:11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Data_Uji_Besar.pdf</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>612.33</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>F73CDD64854D6D70FED675F9D79FD9D8</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>5.3399</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:10:15</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Kesehatan_1.docx</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>13.64</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2BDAEF669A2FAD1BDEB792D063AA61FD</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:10:38</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Kesehatan_2.docx</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>73.03</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>586596B32EE759452CB4B54FF40453D0</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.6741</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:10:40</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Kesehatan_3.docx</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>22.28</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>7830E71273182AE4109F641856417473</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.4992</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-05-16 08:10:41</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>AES-128-BASELINE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Kesehatan.docx</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>85.61</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>27CF574169AF9617DE0D42986575A6AF</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1.1845</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>